<commit_message>
add nl1km day after tomorrow
</commit_message>
<xml_diff>
--- a/cron/planning_rasp_server.xlsx
+++ b/cron/planning_rasp_server.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="995" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="987" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId2"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t xml:space="preserve">type</t>
   </si>
@@ -74,6 +74,9 @@
   </si>
   <si>
     <t xml:space="preserve">NL1KM.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NL1kM.2</t>
   </si>
 </sst>
 </file>
@@ -210,15 +213,15 @@
   <dimension ref="A4:T14"/>
   <sheetFormatPr defaultRowHeight="12.8"/>
   <cols>
-    <col collapsed="false" hidden="false" max="1" min="1" style="0" width="13.6326530612245"/>
-    <col collapsed="false" hidden="false" max="2" min="2" style="0" width="8.50510204081633"/>
-    <col collapsed="false" hidden="false" max="3" min="3" style="0" width="7.96428571428571"/>
-    <col collapsed="false" hidden="false" max="4" min="4" style="0" width="8.50510204081633"/>
-    <col collapsed="false" hidden="false" max="5" min="5" style="0" width="12.8265306122449"/>
-    <col collapsed="false" hidden="false" max="10" min="6" style="0" width="8.50510204081633"/>
-    <col collapsed="false" hidden="false" max="11" min="11" style="0" width="8.18877551020408"/>
-    <col collapsed="false" hidden="false" max="12" min="12" style="0" width="7.1530612244898"/>
-    <col collapsed="false" hidden="false" max="1025" min="13" style="0" width="8.50510204081633"/>
+    <col collapsed="false" hidden="false" max="1" min="1" style="0" width="13.3622448979592"/>
+    <col collapsed="false" hidden="false" max="2" min="2" style="0" width="8.36734693877551"/>
+    <col collapsed="false" hidden="false" max="3" min="3" style="0" width="7.83163265306122"/>
+    <col collapsed="false" hidden="false" max="4" min="4" style="0" width="8.36734693877551"/>
+    <col collapsed="false" hidden="false" max="5" min="5" style="0" width="12.6887755102041"/>
+    <col collapsed="false" hidden="false" max="10" min="6" style="0" width="8.36734693877551"/>
+    <col collapsed="false" hidden="false" max="11" min="11" style="0" width="7.96428571428571"/>
+    <col collapsed="false" hidden="false" max="12" min="12" style="0" width="7.02040816326531"/>
+    <col collapsed="false" hidden="false" max="1025" min="13" style="0" width="8.36734693877551"/>
   </cols>
   <sheetData>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -419,24 +422,26 @@
         <v>0.73975</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">0.33</f>
-        <v>0.33</v>
+        <f aca="false">0.33+3.33</f>
+        <v>3.66</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="4"/>
+      <c r="G10" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="6" t="n">
         <f aca="false">D10+E10/24</f>
-        <v>0.7535</v>
+        <v>0.89225</v>
       </c>
       <c r="M10" s="6" t="n">
         <f aca="false">D12-L10</f>
-        <v>0.23625</v>
+        <v>0.0975</v>
       </c>
       <c r="N10" s="6"/>
       <c r="O10" s="6"/>
@@ -533,7 +538,7 @@
       <c r="D14" s="4"/>
       <c r="E14" s="7" t="n">
         <f aca="false">SUM(E6:E12)</f>
-        <v>12.3</v>
+        <v>15.63</v>
       </c>
       <c r="F14" s="4"/>
       <c r="G14" s="4"/>

</xml_diff>